<commit_message>
Zoeken improved bus plan
</commit_message>
<xml_diff>
--- a/Improved_plan_Feasibility_and_KPI_results.xlsx
+++ b/Improved_plan_Feasibility_and_KPI_results.xlsx
@@ -602,7 +602,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>3837.4404</v>
+        <v>3830.6004</v>
       </c>
     </row>
     <row r="3">
@@ -612,7 +612,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>3197867</v>
+        <v>3192167</v>
       </c>
     </row>
     <row r="4">
@@ -622,7 +622,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>3197.867</v>
+        <v>3192.167</v>
       </c>
     </row>
     <row r="5">
@@ -632,7 +632,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="6">
@@ -642,7 +642,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="7">
@@ -652,7 +652,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>212</v>
+        <v>232</v>
       </c>
     </row>
     <row r="8">
@@ -662,7 +662,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>3.533333333333333</v>
+        <v>3.866666666666667</v>
       </c>
     </row>
     <row r="9">
@@ -672,7 +672,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>9.636363636363637</v>
+        <v>11.6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
899-69-6kbhobhj nhuiiupuohkjlb hbbhkbh u iygigiyoho;owr
</commit_message>
<xml_diff>
--- a/Improved_plan_Feasibility_and_KPI_results.xlsx
+++ b/Improved_plan_Feasibility_and_KPI_results.xlsx
@@ -546,11 +546,11 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Failed</t>
+          <t>Passed</t>
         </is>
       </c>
     </row>
@@ -561,11 +561,11 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>FAILED</t>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -602,7 +602,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>3961.340400000001</v>
+        <v>3830.6004</v>
       </c>
     </row>
     <row r="3">
@@ -612,7 +612,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>3215117</v>
+        <v>3192167</v>
       </c>
     </row>
     <row r="4">
@@ -622,7 +622,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>3215.117</v>
+        <v>3192.167</v>
       </c>
     </row>
     <row r="5">
@@ -632,7 +632,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
     </row>
     <row r="6">
@@ -642,7 +642,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>28</v>
+        <v>13</v>
       </c>
     </row>
     <row r="7">
@@ -652,7 +652,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>148</v>
+        <v>232</v>
       </c>
     </row>
     <row r="8">
@@ -662,7 +662,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>2.466666666666667</v>
+        <v>3.866666666666667</v>
       </c>
     </row>
     <row r="9">
@@ -672,7 +672,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>9.866666666666667</v>
+        <v>11.6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>